<commit_message>
Add terminal/CLI theme (ASCII scene, typed commands, prompt), theme switching, SETUP.md
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -1698,7 +1698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2330,6 +2330,176 @@
       <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Heading on cv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>theme</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Which theme the site opens with: paper (cream, doodles, 3D) or terminal (dark CLI, ASCII). This is what GitHub Pages serves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>theme_toggle</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>yes/no - let visitors switch between the two themes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>terminal_user</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>harsh@portfolio</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Prompt shown in the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>terminal_bg</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>#0b0d10</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Terminal background</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>terminal_fg</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>#d9dee4</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Terminal text</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>terminal_dim</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>#6f7a86</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Terminal muted text</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>terminal_accent</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>#7dd3a0</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Terminal accent (links, prompt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>terminal_accent_2</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>#f2c86b</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Terminal second accent (years, keys)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>terminal_scanlines</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>yes/no - CRT scanline overlay in the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>terminal_font</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>JetBrains Mono</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Any Google monospace font</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Terminal theme rework: black/white/yellow, character field, ASCII wireframe/portrait, boot, shortcuts; ML history moved to history.html
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -491,7 +491,6 @@
           <t>HOW THIS WORKBOOK WORKS</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr"/>
@@ -1698,7 +1697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2392,7 +2391,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>#0b0d10</t>
+          <t>#000000</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -2409,7 +2408,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>#d9dee4</t>
+          <t>#ffffff</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -2426,7 +2425,7 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>#6f7a86</t>
+          <t>#8a8a8a</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
@@ -2443,63 +2442,93 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>#7dd3a0</t>
+          <t>#f2c86b</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Terminal accent (links, prompt)</t>
+          <t>The one accent colour in the terminal theme (yellow): highlights, prompt caret, animation</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>terminal_accent_2</t>
+          <t>terminal_scanlines</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>#f2c86b</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Terminal second accent (years, keys)</t>
+          <t>yes/no - CRT scanline overlay in the terminal theme</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>terminal_scanlines</t>
+          <t>terminal_font</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
+          <t>JetBrains Mono</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Any Google monospace font</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>terminal_history</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>yes/no - CRT scanline overlay in the terminal theme</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>terminal_font</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>JetBrains Mono</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>Any Google monospace font</t>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>yes/no - link to history.html (the ML-history page with the ASCII diagrams) from the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>terminal_boot</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>yes/no - short boot sequence on first load (terminal theme)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>hero_note_terminal</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Optional extra line under the hero in the terminal theme</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make everything workbook-driven: Text sheet for all UI strings, show/hide switches for every part and page, per-section theme/nav/cv flags, deploy prune, studio publish plan, upgrade tool, USER_GUIDE
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -12,15 +12,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sections" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Links" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numbers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Education" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experience" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achievements" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certifications" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contact" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numbers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Education" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experience" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achievements" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certifications" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contact" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +65,10 @@
       <color rgb="00F7EFE1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00F7EFE1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -95,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +115,10 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -478,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -792,12 +801,494 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Text sheet</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Every word the site prints that is not your content (buttons, hints, prompt commands, help text). Change any value; delete a row to get the default back. {placeholders} are filled in by the site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Show / hide</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Settings rows starting with show_ / terminal_ / paper_ switch parts and pages on or off. Sections: themes (all/paper/terminal), show_in_nav, show_in_cv, nav_label, command. Pages switched off are not published.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EFE3CC"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Languages</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Languages</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>JavaScript</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Languages</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>TypeScript</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Languages</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>PyTorch</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Hugging Face</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>PEFT / DoRA</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>vLLM</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Computer Vision</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>pandas / NumPy</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>RAG &amp; document parsing</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>AI / ML</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>FastAPI</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Frameworks</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Django</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Frameworks</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>React</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Frameworks</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>REST APIs</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Frameworks</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Docker</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>nginx</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare Tunnel</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>SQLite</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>NVIDIA DGX</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; tools</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -924,7 +1415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -1274,7 +1765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -1393,7 +1884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -1566,7 +2057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -1697,7 +2188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2525,10 +3016,383 @@
           <t>hero_note_terminal</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>Optional extra line under the hero in the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>show_cv_page</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>yes/no - publish cv.html and link to it</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>show_history_page</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>yes/no - publish history.html (ML history, terminal theme) and link to it</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>show_nav</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>yes/no - top navigation bar (both themes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>show_footer</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>yes/no - footer (paper) / closing line (terminal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>show_scroll_cue</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>yes/no - 'scroll' hint under the hero</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>show_era_note</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>yes/no - the era card on the paper hero</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>show_hero_note</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>yes/no - hero_note lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>show_roles</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>yes/no - the rotating 'I build ...' line</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>show_socials</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>yes/no - social icons/links in the hero</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>show_location</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>yes/no - location in hero and contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>show_availability</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>yes/no - the availability pill/line (also hidden when availability is blank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>show_generated_line</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>yes/no - the small 'generated from content.xlsx' line</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>show_section_numbers</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>yes/no - the '--- 01 ---' dividers in the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>show_status_bar</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>yes/no - shortcut legend at the bottom of the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>show_clock</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>yes/no - clock + uptime in the terminal status bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>show_prompt</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>yes/no - the typeable command prompt in the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>show_shortcuts</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>yes/no - single-key shortcuts h/p/c/i/?/ in the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>terminal_field</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>yes/no - animated character field behind the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>terminal_wireframe</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>yes/no - rotating ASCII wireframe / portrait on the right</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>terminal_banner</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ascii</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ascii / text / none - how the name is shown in the terminal hero</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>terminal_typing</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>yes/no - typed commands and line-by-line printing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>paper_modal</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>yes/no - clicking a project card opens the detail modal (paper theme)</t>
         </is>
       </c>
     </row>
@@ -2544,7 +3408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2559,6 +3423,11 @@
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2622,6 +3491,31 @@
           <t>cta_link</t>
         </is>
       </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>themes</t>
+        </is>
+      </c>
+      <c r="N1" s="8" t="inlineStr">
+        <is>
+          <t>show_in_nav</t>
+        </is>
+      </c>
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>show_in_cv</t>
+        </is>
+      </c>
+      <c r="P1" s="8" t="inlineStr">
+        <is>
+          <t>nav_label</t>
+        </is>
+      </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>command</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -2666,6 +3560,21 @@
       </c>
       <c r="K2" s="6" t="inlineStr"/>
       <c r="L2" s="6" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -2714,6 +3623,21 @@
       </c>
       <c r="K3" s="6" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2758,6 +3682,21 @@
       </c>
       <c r="K4" s="6" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2806,6 +3745,21 @@
       </c>
       <c r="K5" s="6" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2850,6 +3804,21 @@
       </c>
       <c r="K6" s="6" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2910,6 +3879,21 @@
           <t>https://github.com/Harsh4-Dev</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2954,6 +3938,21 @@
       </c>
       <c r="K8" s="6" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -3002,6 +4001,21 @@
       </c>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -3050,9 +4064,24 @@
       </c>
       <c r="K10" s="6" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a valid value" error="Pick one of: timeline, cards, tags, stats, text, list, gallery, table, contact" type="list">
       <formula1>"timeline,cards,tags,stats,text,list,gallery,table,contact"</formula1>
     </dataValidation>
@@ -3060,6 +4089,15 @@
       <formula1>"neuron,perceptron,mlp,cnn,deep,transformer,constellation"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a valid value" error="Pick one of: yes, no" type="list">
+      <formula1>"yes,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"all,paper,terminal"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"yes,no"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3074,7 +4112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3122,6 +4160,11 @@
           <t>order</t>
         </is>
       </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -3157,6 +4200,11 @@
       <c r="G2" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -3192,6 +4240,11 @@
       <c r="G3" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3227,6 +4280,11 @@
       <c r="G4" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3262,6 +4320,11 @@
       <c r="G5" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3297,6 +4360,11 @@
       <c r="G6" s="6" t="n">
         <v>5</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3332,6 +4400,11 @@
       <c r="G7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3366,6 +4439,11 @@
       </c>
       <c r="G8" s="6" t="n">
         <v>7</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3510,6 +4588,913 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="006B6FD6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>paper_hero_scroll</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>scroll</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Label under the scroll cue</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>paper_card_more</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>read more</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Link text on project cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>paper_link_open</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Default label for a row's main link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>paper_footer_cv</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>CV page</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Footer link to cv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>paper_footer_top</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Back to top ↑</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>paper_footer_copyright</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>© {year} {name}.</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Placeholders: {year} {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>paper_footer_generated</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Content generated from {source} on {date}.</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Placeholders: {source} {date}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>paper_empty_section</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Nothing here yet — add rows to the '{id}' sheet.</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>paper_theme_toggle</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Header button that switches to the terminal theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>paper_menu</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Mobile menu button label (accessibility)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>paper_skip</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Skip to content</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>paper_loading</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>warming up the perceptron</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Shown while content.json loads</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>paper_modal_close</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>cv_back</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>← Portfolio</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Button on cv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>cv_print</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Print / Save as PDF</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>cv_tools</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Tools:</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Label before a row's tags on cv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>cv_generated</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Generated from {source} · {date}</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>term_title</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>{user}:~/portfolio</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Window title, top-left</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>term_menu</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>menu</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Mobile menu button</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>term_tab_history</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Tab label</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>term_tab_cv</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>cv</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Tab label</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>term_tab_paper</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Theme switch tab label</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>term_whoami</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>whoami</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Command shown above the name</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>term_scroll_hint</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>▼ scroll · ? for shortcuts · / to type a command</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>term_resume</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>resume.pdf</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Link label for resume_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>term_cv_link</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>cv</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Link label for cv.html in the hero</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>term_boot_cmd</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>./portfolio --serve</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>First boot line</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>term_boot_lines</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>[ ok ] reading {source} ........ {items} items | [ ok ] mounting sections ........... {sections} | [ ok ] font grid ................... {grid} | [ ok ] warming up the wireframe</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Boot lines separated by |. Placeholders: {source} {items} {sections} {grid}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>term_total</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>total {n}</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>First line of a project listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>term_tags</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>tags:</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>term_readme</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>cat {name}/README.md</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Command shown when a project is expanded</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_text</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>cat {id}.md</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Command for text sections ({id} = sheet name, lowercase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_stats</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>./{id} --summary</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_timeline</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>cat {id}.log</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_cards</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>ls -la {id}/</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_tags</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>tree {id}/</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_list</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>cat {id}.txt</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_gallery</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>ls {id}/*.png</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_table</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>column -t {id}.tsv</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>term_cmd_contact</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>cat contact.txt</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>term_prompt_placeholder</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>help</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>term_keys</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>h:home; p:projects; c:contact; i:invert; /:prompt; ?:help</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Status bar legend, key:label pairs separated by ;</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>term_help</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>ls · cat &lt;section&gt; · open &lt;project|n&gt; · history · invert · theme paper · cv · email · top · clear</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Printed by help / ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>term_not_found</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>bash: {cmd}: command not found (try help)</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>term_no_such_file</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>cat: {arg}: no such file or directory</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>term_no_match</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>open: nothing matches '{arg}' — projects: {list}</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>term_opening</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>opening {title} …</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>term_goto</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>→ {title}</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>term_sudo</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>nice try.</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>term_exit</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>there is no escape. try theme paper.</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>term_empty_section</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>{id}: no entries yet — add rows to the '{sheet}' sheet</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>term_generated</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>{note} — generated from {source} · {date}</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Closing line. Placeholders: {note} = footer_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>term_uptime</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>up {m}m{s}s</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>hist_cmd</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>cat history.md</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Command line at the top of history.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>hist_hint</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>every diagram is a real architecture. ↑ ↓ or click to switch, it dissolves into dust and the next one condenses.</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>hist_tab_portfolio</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>portfolio</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>hist_tab_paper</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>hist_path</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>~/history</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>Shown after the user name in the title</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00EFE3CC"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3568,7 +5553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -3691,7 +5676,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EFE3CC"/>
@@ -3886,461 +5871,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00EFE3CC"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>group</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>level</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Python</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Languages</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>SQL</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Languages</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>JavaScript</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Languages</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>TypeScript</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Languages</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>PyTorch</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Hugging Face</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>PEFT / DoRA</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>vLLM</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>LangChain</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Computer Vision</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>pandas / NumPy</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>RAG &amp; document parsing</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>AI / ML</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>FastAPI</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Frameworks</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Django</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Frameworks</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>React</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Frameworks</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>REST APIs</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Frameworks</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Docker</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Linux</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>nginx</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Git</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Cloudflare Tunnel</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>SQLite</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>NVIDIA DGX</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; tools</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Serve the terminal theme only: lock the theme when the toggle is off, add generated theme-boot.js
- Settings: theme = terminal, theme_toggle = no
- resolveTheme ignores ?theme= and the visitor's saved choice when switching is disabled
- build_content writes site/assets/js/theme-boot.js so the first paint uses the terminal
  background instead of flashing the paper cream

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -801,7 +801,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -2831,7 +2830,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>paper</t>
+          <t>terminal</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -2848,7 +2847,7 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Remove the CV page, resume PDF, phone and location from the published site
- Settings: show_cv_page = no, location and phone cleared, show_location = no, resume_url cleared,
  and the "Download CV" call to action removed
- site/cv.html, site/assets/js/cv.js and the resume PDF moved to private/, which is gitignored,
  so they stay on disk but are neither committed nor deployed
- tools/make_seed.py no longer carries the location or the resume path as starter defaults

Note: earlier commits still contain the PDF and the location, so the history needs rewriting or
the repository recreating for these to be genuinely private.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -2371,11 +2371,7 @@
           <t>location</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Trichy, Tamil Nadu, India</t>
-        </is>
-      </c>
+      <c r="B11" s="7" t="inlineStr"/>
       <c r="C11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -2423,11 +2419,7 @@
           <t>resume_url</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>assets/Harshavardhan-S-Resume.pdf</t>
-        </is>
-      </c>
+      <c r="B15" s="7" t="inlineStr"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
           <t>PDF path or URL for the CV button (blank = use cv.html)</t>
@@ -2470,11 +2462,7 @@
           <t>secondary_cta_label</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Download CV</t>
-        </is>
-      </c>
+      <c r="B18" s="7" t="inlineStr"/>
       <c r="C18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
@@ -2483,11 +2471,7 @@
           <t>secondary_cta_link</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>cv.html</t>
-        </is>
-      </c>
+      <c r="B19" s="7" t="inlineStr"/>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
@@ -3029,7 +3013,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3182,7 +3166,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">

</xml_diff>